<commit_message>
thực hiện automation testing cho modul chức năng quản lý giao hàng admin_shipment
</commit_message>
<xml_diff>
--- a/23130064_TruongCaoDoan/Group13_23130064_TruongCaoDoan.xlsx
+++ b/23130064_TruongCaoDoan/Group13_23130064_TruongCaoDoan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\n4k1\test\gh\Tester\23130064_TruongCaoDoan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5729AB16-8877-4CE7-8D51-9C1DF6067D12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B7327B-A903-47F7-9CE7-67A727CB3690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="475">
   <si>
     <t>TEST CASE SPECIFICATION</t>
   </si>
@@ -612,9 +612,6 @@
     <t>1. Bảng dữ liệu chỉ hiển thị các đơn hàng đã bị hủy (Cancelled).</t>
   </si>
   <si>
-    <t>Kiểm tra lọc danh sách giao hàng theo Quốc gia / Tỉnh thành</t>
-  </si>
-  <si>
     <t>admin_ord_12</t>
   </si>
   <si>
@@ -1101,11 +1098,6 @@
 2. Click nút [Change status]
 3. Chọn 'Complete'  
 4. Click [Save]</t>
-  </si>
-  <si>
-    <t>Step:
-1. Chọn Country = [United States]
-2. Click nút [Search]</t>
   </si>
   <si>
     <t>1. HIển thị list trạng thái có thể thay đổi gồm "Complete"
@@ -1678,6 +1670,26 @@
   <si>
     <t>Không hiển thị thông báo nhập số giá sản phẩm lớn hơn không.
 Hệ thống thực hiện lưu giá sản phẩm là âm trong đơn hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiểm tra lọc danh sách giao hàng theo Quốc gia </t>
+  </si>
+  <si>
+    <t>Kiểm tra lọc danh sách giao hàng theo Quốc gia</t>
+  </si>
+  <si>
+    <t>Step:
+1. Chọn Country = [United States of America]
+2. Click nút [Search]</t>
+  </si>
+  <si>
+    <t>Do đơn hàng không đủ nhiều để thực hiện chuyển trang</t>
+  </si>
+  <si>
+    <t>Do chuyển trang kế tiếp không được nên không thể thực hiện được test case này</t>
+  </si>
+  <si>
+    <t>Thực tế hệ thống tiến hành tìm kiếm chứ không thông báo ngày nhận không hợp lệ</t>
   </si>
 </sst>
 </file>
@@ -1943,6 +1955,9 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1952,9 +1967,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2184,14 +2196,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
     </row>
     <row r="4" spans="2:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
@@ -3294,13 +3306,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
     </row>
     <row r="4" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
@@ -4424,7 +4436,7 @@
       <c r="B2" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="C2" s="30" t="s">
         <v>57</v>
       </c>
       <c r="D2" s="9" t="s">
@@ -4438,7 +4450,7 @@
     <row r="3" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
-      <c r="C3" s="30"/>
+      <c r="C3" s="31"/>
       <c r="D3" s="9" t="s">
         <v>64</v>
       </c>
@@ -4450,7 +4462,7 @@
     <row r="4" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
-      <c r="C4" s="31"/>
+      <c r="C4" s="32"/>
       <c r="D4" s="9" t="s">
         <v>67</v>
       </c>
@@ -4462,7 +4474,7 @@
     <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="30" t="s">
         <v>68</v>
       </c>
       <c r="D5" s="9" t="s">
@@ -4476,7 +4488,7 @@
     <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
-      <c r="C6" s="30"/>
+      <c r="C6" s="31"/>
       <c r="D6" s="9" t="s">
         <v>71</v>
       </c>
@@ -4488,7 +4500,7 @@
     <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
-      <c r="C7" s="30"/>
+      <c r="C7" s="31"/>
       <c r="D7" s="9" t="s">
         <v>72</v>
       </c>
@@ -4500,7 +4512,7 @@
     <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
-      <c r="C8" s="31"/>
+      <c r="C8" s="32"/>
       <c r="D8" s="9" t="s">
         <v>73</v>
       </c>
@@ -4512,7 +4524,7 @@
     <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="30" t="s">
         <v>74</v>
       </c>
       <c r="D9" s="9" t="s">
@@ -4526,7 +4538,7 @@
     <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
-      <c r="C10" s="30"/>
+      <c r="C10" s="31"/>
       <c r="D10" s="9" t="s">
         <v>76</v>
       </c>
@@ -4538,7 +4550,7 @@
     <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
-      <c r="C11" s="30"/>
+      <c r="C11" s="31"/>
       <c r="D11" s="9" t="s">
         <v>77</v>
       </c>
@@ -4550,7 +4562,7 @@
     <row r="12" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
-      <c r="C12" s="30"/>
+      <c r="C12" s="31"/>
       <c r="D12" s="9" t="s">
         <v>78</v>
       </c>
@@ -4562,7 +4574,7 @@
     <row r="13" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
-      <c r="C13" s="30"/>
+      <c r="C13" s="31"/>
       <c r="D13" s="9" t="s">
         <v>79</v>
       </c>
@@ -4574,7 +4586,7 @@
     <row r="14" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
-      <c r="C14" s="30"/>
+      <c r="C14" s="31"/>
       <c r="D14" s="9" t="s">
         <v>80</v>
       </c>
@@ -4586,7 +4598,7 @@
     <row r="15" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
-      <c r="C15" s="30"/>
+      <c r="C15" s="31"/>
       <c r="D15" s="9" t="s">
         <v>81</v>
       </c>
@@ -4598,7 +4610,7 @@
     <row r="16" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
-      <c r="C16" s="30"/>
+      <c r="C16" s="31"/>
       <c r="D16" s="9" t="s">
         <v>82</v>
       </c>
@@ -4610,7 +4622,7 @@
     <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
-      <c r="C17" s="30"/>
+      <c r="C17" s="31"/>
       <c r="D17" s="9" t="s">
         <v>83</v>
       </c>
@@ -4622,7 +4634,7 @@
     <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
-      <c r="C18" s="30"/>
+      <c r="C18" s="31"/>
       <c r="D18" s="9" t="s">
         <v>84</v>
       </c>
@@ -4634,7 +4646,7 @@
     <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
-      <c r="C19" s="30"/>
+      <c r="C19" s="31"/>
       <c r="D19" s="9" t="s">
         <v>85</v>
       </c>
@@ -4646,7 +4658,7 @@
     <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
-      <c r="C20" s="30"/>
+      <c r="C20" s="31"/>
       <c r="D20" s="9" t="s">
         <v>86</v>
       </c>
@@ -4658,7 +4670,7 @@
     <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
-      <c r="C21" s="31"/>
+      <c r="C21" s="32"/>
       <c r="D21" s="9" t="s">
         <v>87</v>
       </c>
@@ -4670,7 +4682,7 @@
     <row r="22" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="30" t="s">
         <v>88</v>
       </c>
       <c r="D22" s="9" t="s">
@@ -4684,7 +4696,7 @@
     <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
-      <c r="C23" s="30"/>
+      <c r="C23" s="31"/>
       <c r="D23" s="9" t="s">
         <v>90</v>
       </c>
@@ -4696,7 +4708,7 @@
     <row r="24" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
-      <c r="C24" s="30"/>
+      <c r="C24" s="31"/>
       <c r="D24" s="9" t="s">
         <v>91</v>
       </c>
@@ -4708,7 +4720,7 @@
     <row r="25" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
-      <c r="C25" s="31"/>
+      <c r="C25" s="32"/>
       <c r="D25" s="9" t="s">
         <v>92</v>
       </c>
@@ -4720,7 +4732,7 @@
     <row r="26" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="30" t="s">
         <v>93</v>
       </c>
       <c r="D26" s="9" t="s">
@@ -4734,7 +4746,7 @@
     <row r="27" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
-      <c r="C27" s="30"/>
+      <c r="C27" s="31"/>
       <c r="D27" s="9" t="s">
         <v>95</v>
       </c>
@@ -4746,7 +4758,7 @@
     <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
-      <c r="C28" s="31"/>
+      <c r="C28" s="32"/>
       <c r="D28" s="9" t="s">
         <v>96</v>
       </c>
@@ -4758,7 +4770,7 @@
     <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
-      <c r="C29" s="29" t="s">
+      <c r="C29" s="30" t="s">
         <v>97</v>
       </c>
       <c r="D29" s="9" t="s">
@@ -4772,7 +4784,7 @@
     <row r="30" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
-      <c r="C30" s="31"/>
+      <c r="C30" s="32"/>
       <c r="D30" s="9" t="s">
         <v>99</v>
       </c>
@@ -4784,7 +4796,7 @@
     <row r="31" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
-      <c r="C31" s="29" t="s">
+      <c r="C31" s="30" t="s">
         <v>100</v>
       </c>
       <c r="D31" s="9" t="s">
@@ -4798,7 +4810,7 @@
     <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
-      <c r="C32" s="30"/>
+      <c r="C32" s="31"/>
       <c r="D32" s="9" t="s">
         <v>104</v>
       </c>
@@ -4810,7 +4822,7 @@
     <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
-      <c r="C33" s="31"/>
+      <c r="C33" s="32"/>
       <c r="D33" s="9" t="s">
         <v>109</v>
       </c>
@@ -4822,7 +4834,7 @@
     <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
-      <c r="C34" s="29" t="s">
+      <c r="C34" s="30" t="s">
         <v>111</v>
       </c>
       <c r="D34" s="9" t="s">
@@ -4836,7 +4848,7 @@
     <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
-      <c r="C35" s="30"/>
+      <c r="C35" s="31"/>
       <c r="D35" s="9" t="s">
         <v>115</v>
       </c>
@@ -4848,7 +4860,7 @@
     <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
-      <c r="C36" s="31"/>
+      <c r="C36" s="32"/>
       <c r="D36" s="9" t="s">
         <v>118</v>
       </c>
@@ -4860,7 +4872,7 @@
     <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
-      <c r="C37" s="29" t="s">
+      <c r="C37" s="30" t="s">
         <v>120</v>
       </c>
       <c r="D37" s="9" t="s">
@@ -4874,7 +4886,7 @@
     <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" s="9"/>
       <c r="B38" s="9"/>
-      <c r="C38" s="30"/>
+      <c r="C38" s="31"/>
       <c r="D38" s="9" t="s">
         <v>125</v>
       </c>
@@ -4886,7 +4898,7 @@
     <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" s="9"/>
       <c r="B39" s="9"/>
-      <c r="C39" s="31"/>
+      <c r="C39" s="32"/>
       <c r="D39" s="9" t="s">
         <v>127</v>
       </c>
@@ -4898,7 +4910,7 @@
     <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A40" s="9"/>
       <c r="B40" s="9"/>
-      <c r="C40" s="29" t="s">
+      <c r="C40" s="30" t="s">
         <v>130</v>
       </c>
       <c r="D40" s="9" t="s">
@@ -4912,7 +4924,7 @@
     <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
-      <c r="C41" s="30"/>
+      <c r="C41" s="31"/>
       <c r="D41" s="9" t="s">
         <v>133</v>
       </c>
@@ -4924,7 +4936,7 @@
     <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A42" s="9"/>
       <c r="B42" s="9"/>
-      <c r="C42" s="30"/>
+      <c r="C42" s="31"/>
       <c r="D42" s="9" t="s">
         <v>135</v>
       </c>
@@ -4936,7 +4948,7 @@
     <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A43" s="9"/>
       <c r="B43" s="9"/>
-      <c r="C43" s="31"/>
+      <c r="C43" s="32"/>
       <c r="D43" s="9" t="s">
         <v>139</v>
       </c>
@@ -4948,7 +4960,7 @@
     <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A44" s="9"/>
       <c r="B44" s="9"/>
-      <c r="C44" s="29" t="s">
+      <c r="C44" s="30" t="s">
         <v>141</v>
       </c>
       <c r="D44" s="9" t="s">
@@ -4962,7 +4974,7 @@
     <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A45" s="9"/>
       <c r="B45" s="9"/>
-      <c r="C45" s="31"/>
+      <c r="C45" s="32"/>
       <c r="D45" s="9" t="s">
         <v>148</v>
       </c>
@@ -4976,7 +4988,7 @@
       <c r="B46" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="C46" s="29" t="s">
+      <c r="C46" s="30" t="s">
         <v>57</v>
       </c>
       <c r="D46" s="9" t="s">
@@ -4990,7 +5002,7 @@
     <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A47" s="9"/>
       <c r="B47" s="9"/>
-      <c r="C47" s="31"/>
+      <c r="C47" s="32"/>
       <c r="D47" s="9" t="s">
         <v>158</v>
       </c>
@@ -5002,7 +5014,7 @@
     <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A48" s="9"/>
       <c r="B48" s="9"/>
-      <c r="C48" s="29" t="s">
+      <c r="C48" s="30" t="s">
         <v>162</v>
       </c>
       <c r="D48" s="9" t="s">
@@ -5016,7 +5028,7 @@
     <row r="49" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A49" s="9"/>
       <c r="B49" s="9"/>
-      <c r="C49" s="30"/>
+      <c r="C49" s="31"/>
       <c r="D49" s="9" t="s">
         <v>174</v>
       </c>
@@ -5028,9 +5040,9 @@
     <row r="50" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A50" s="9"/>
       <c r="B50" s="9"/>
-      <c r="C50" s="30"/>
+      <c r="C50" s="31"/>
       <c r="D50" s="9" t="s">
-        <v>179</v>
+        <v>470</v>
       </c>
       <c r="E50" s="15" t="s">
         <v>70</v>
@@ -5040,9 +5052,9 @@
     <row r="51" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A51" s="9"/>
       <c r="B51" s="9"/>
-      <c r="C51" s="30"/>
+      <c r="C51" s="31"/>
       <c r="D51" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E51" s="15" t="s">
         <v>70</v>
@@ -5052,9 +5064,9 @@
     <row r="52" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A52" s="9"/>
       <c r="B52" s="9"/>
-      <c r="C52" s="30"/>
+      <c r="C52" s="31"/>
       <c r="D52" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E52" s="15" t="s">
         <v>70</v>
@@ -5064,9 +5076,9 @@
     <row r="53" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A53" s="9"/>
       <c r="B53" s="9"/>
-      <c r="C53" s="30"/>
+      <c r="C53" s="31"/>
       <c r="D53" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E53" s="15" t="s">
         <v>70</v>
@@ -5076,9 +5088,9 @@
     <row r="54" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A54" s="9"/>
       <c r="B54" s="9"/>
-      <c r="C54" s="31"/>
+      <c r="C54" s="32"/>
       <c r="D54" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E54" s="15" t="s">
         <v>70</v>
@@ -5088,11 +5100,11 @@
     <row r="55" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A55" s="9"/>
       <c r="B55" s="9"/>
-      <c r="C55" s="29" t="s">
-        <v>197</v>
+      <c r="C55" s="30" t="s">
+        <v>196</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E55" s="15" t="s">
         <v>70</v>
@@ -5102,9 +5114,9 @@
     <row r="56" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A56" s="9"/>
       <c r="B56" s="9"/>
-      <c r="C56" s="31"/>
+      <c r="C56" s="32"/>
       <c r="D56" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E56" s="15" t="s">
         <v>70</v>
@@ -5114,11 +5126,11 @@
     <row r="57" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A57" s="9"/>
       <c r="B57" s="9"/>
-      <c r="C57" s="29" t="s">
+      <c r="C57" s="30" t="s">
+        <v>204</v>
+      </c>
+      <c r="D57" s="9" t="s">
         <v>205</v>
-      </c>
-      <c r="D57" s="9" t="s">
-        <v>206</v>
       </c>
       <c r="E57" s="15" t="s">
         <v>70</v>
@@ -5128,9 +5140,9 @@
     <row r="58" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A58" s="9"/>
       <c r="B58" s="9"/>
-      <c r="C58" s="30"/>
+      <c r="C58" s="31"/>
       <c r="D58" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E58" s="15" t="s">
         <v>70</v>
@@ -5140,9 +5152,9 @@
     <row r="59" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A59" s="9"/>
       <c r="B59" s="9"/>
-      <c r="C59" s="30"/>
+      <c r="C59" s="31"/>
       <c r="D59" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E59" s="15" t="s">
         <v>70</v>
@@ -5152,9 +5164,9 @@
     <row r="60" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A60" s="9"/>
       <c r="B60" s="9"/>
-      <c r="C60" s="30"/>
+      <c r="C60" s="31"/>
       <c r="D60" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E60" s="15" t="s">
         <v>70</v>
@@ -5164,9 +5176,9 @@
     <row r="61" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A61" s="9"/>
       <c r="B61" s="9"/>
-      <c r="C61" s="30"/>
+      <c r="C61" s="31"/>
       <c r="D61" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E61" s="15" t="s">
         <v>70</v>
@@ -5176,9 +5188,9 @@
     <row r="62" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A62" s="9"/>
       <c r="B62" s="9"/>
-      <c r="C62" s="31"/>
+      <c r="C62" s="32"/>
       <c r="D62" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E62" s="15" t="s">
         <v>70</v>
@@ -5188,11 +5200,11 @@
     <row r="63" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A63" s="9"/>
       <c r="B63" s="9"/>
-      <c r="C63" s="29" t="s">
-        <v>220</v>
+      <c r="C63" s="30" t="s">
+        <v>219</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E63" s="15" t="s">
         <v>70</v>
@@ -5202,9 +5214,9 @@
     <row r="64" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A64" s="9"/>
       <c r="B64" s="9"/>
-      <c r="C64" s="30"/>
+      <c r="C64" s="31"/>
       <c r="D64" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E64" s="15" t="s">
         <v>70</v>
@@ -5214,9 +5226,9 @@
     <row r="65" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A65" s="9"/>
       <c r="B65" s="9"/>
-      <c r="C65" s="31"/>
+      <c r="C65" s="32"/>
       <c r="D65" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E65" s="15" t="s">
         <v>70</v>
@@ -5226,13 +5238,13 @@
     <row r="66" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A66" s="9"/>
       <c r="B66" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="C66" s="29" t="s">
-        <v>235</v>
+        <v>232</v>
+      </c>
+      <c r="C66" s="30" t="s">
+        <v>234</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E66" s="14" t="s">
         <v>60</v>
@@ -5242,9 +5254,9 @@
     <row r="67" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A67" s="9"/>
       <c r="B67" s="9"/>
-      <c r="C67" s="30"/>
+      <c r="C67" s="31"/>
       <c r="D67" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E67" s="15" t="s">
         <v>70</v>
@@ -5254,9 +5266,9 @@
     <row r="68" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A68" s="9"/>
       <c r="B68" s="9"/>
-      <c r="C68" s="30"/>
+      <c r="C68" s="31"/>
       <c r="D68" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E68" s="15" t="s">
         <v>70</v>
@@ -5266,9 +5278,9 @@
     <row r="69" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A69" s="9"/>
       <c r="B69" s="9"/>
-      <c r="C69" s="30"/>
+      <c r="C69" s="31"/>
       <c r="D69" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E69" s="15" t="s">
         <v>70</v>
@@ -5278,9 +5290,9 @@
     <row r="70" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A70" s="9"/>
       <c r="B70" s="9"/>
-      <c r="C70" s="30"/>
+      <c r="C70" s="31"/>
       <c r="D70" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E70" s="15" t="s">
         <v>70</v>
@@ -5290,9 +5302,9 @@
     <row r="71" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A71" s="9"/>
       <c r="B71" s="9"/>
-      <c r="C71" s="31"/>
+      <c r="C71" s="32"/>
       <c r="D71" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E71" s="15" t="s">
         <v>70</v>
@@ -5302,11 +5314,11 @@
     <row r="72" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A72" s="9"/>
       <c r="B72" s="9"/>
-      <c r="C72" s="29" t="s">
-        <v>255</v>
+      <c r="C72" s="30" t="s">
+        <v>254</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E72" s="15" t="s">
         <v>70</v>
@@ -5316,9 +5328,9 @@
     <row r="73" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A73" s="9"/>
       <c r="B73" s="9"/>
-      <c r="C73" s="30"/>
+      <c r="C73" s="31"/>
       <c r="D73" s="9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E73" s="15" t="s">
         <v>70</v>
@@ -5328,9 +5340,9 @@
     <row r="74" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A74" s="9"/>
       <c r="B74" s="9"/>
-      <c r="C74" s="30"/>
+      <c r="C74" s="31"/>
       <c r="D74" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E74" s="15" t="s">
         <v>70</v>
@@ -5340,9 +5352,9 @@
     <row r="75" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A75" s="9"/>
       <c r="B75" s="9"/>
-      <c r="C75" s="30"/>
+      <c r="C75" s="31"/>
       <c r="D75" s="9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E75" s="15" t="s">
         <v>70</v>
@@ -5352,9 +5364,9 @@
     <row r="76" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A76" s="9"/>
       <c r="B76" s="9"/>
-      <c r="C76" s="31"/>
+      <c r="C76" s="32"/>
       <c r="D76" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E76" s="15" t="s">
         <v>70</v>
@@ -5364,11 +5376,11 @@
     <row r="77" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A77" s="9"/>
       <c r="B77" s="9"/>
-      <c r="C77" s="29" t="s">
-        <v>272</v>
+      <c r="C77" s="30" t="s">
+        <v>271</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E77" s="15" t="s">
         <v>70</v>
@@ -5378,9 +5390,9 @@
     <row r="78" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A78" s="9"/>
       <c r="B78" s="9"/>
-      <c r="C78" s="30"/>
+      <c r="C78" s="31"/>
       <c r="D78" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E78" s="15" t="s">
         <v>70</v>
@@ -5390,9 +5402,9 @@
     <row r="79" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A79" s="9"/>
       <c r="B79" s="9"/>
-      <c r="C79" s="30"/>
+      <c r="C79" s="31"/>
       <c r="D79" s="9" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E79" s="15" t="s">
         <v>70</v>
@@ -5402,9 +5414,9 @@
     <row r="80" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A80" s="9"/>
       <c r="B80" s="9"/>
-      <c r="C80" s="31"/>
+      <c r="C80" s="32"/>
       <c r="D80" s="9" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E80" s="15" t="s">
         <v>70</v>
@@ -5414,11 +5426,11 @@
     <row r="81" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A81" s="9"/>
       <c r="B81" s="9"/>
-      <c r="C81" s="29" t="s">
-        <v>290</v>
+      <c r="C81" s="30" t="s">
+        <v>289</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E81" s="15" t="s">
         <v>70</v>
@@ -5428,9 +5440,9 @@
     <row r="82" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A82" s="9"/>
       <c r="B82" s="9"/>
-      <c r="C82" s="31"/>
+      <c r="C82" s="32"/>
       <c r="D82" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E82" s="15" t="s">
         <v>70</v>
@@ -5441,10 +5453,10 @@
       <c r="A83" s="9"/>
       <c r="B83" s="9"/>
       <c r="C83" s="12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E83" s="15" t="s">
         <v>70</v>
@@ -5455,10 +5467,10 @@
       <c r="A84" s="9"/>
       <c r="B84" s="9"/>
       <c r="C84" s="22" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E84" s="15" t="s">
         <v>70</v>
@@ -5469,10 +5481,10 @@
       <c r="A85" s="9"/>
       <c r="B85" s="9"/>
       <c r="C85" s="23" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D85" s="9" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="E85" s="15" t="s">
         <v>70</v>
@@ -6396,6 +6408,16 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="C9:C21"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="C57:C62"/>
+    <mergeCell ref="C63:C65"/>
+    <mergeCell ref="C66:C71"/>
     <mergeCell ref="C72:C76"/>
     <mergeCell ref="C77:C80"/>
     <mergeCell ref="C81:C82"/>
@@ -6406,16 +6428,6 @@
     <mergeCell ref="C46:C47"/>
     <mergeCell ref="C48:C54"/>
     <mergeCell ref="C55:C56"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="C57:C62"/>
-    <mergeCell ref="C63:C65"/>
-    <mergeCell ref="C66:C71"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="C5:C8"/>
-    <mergeCell ref="C9:C21"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="C26:C28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -6485,7 +6497,7 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="16">
         <f>COUNTIF(F9:F52, "Passed")</f>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B6" s="17">
         <f>COUNTIF(F9:F52, "Failed")</f>
@@ -6497,7 +6509,7 @@
       </c>
       <c r="D6" s="19">
         <f>COUNTIF(F9:F52, "Blocked")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" s="20">
         <f>COUNTIF(F9:F52, "Skipped")</f>
@@ -6553,7 +6565,7 @@
       <c r="F9" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="27">
         <v>46323</v>
       </c>
       <c r="H9" s="9"/>
@@ -6577,7 +6589,7 @@
       <c r="F10" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G10" s="32">
+      <c r="G10" s="27">
         <v>46324</v>
       </c>
       <c r="H10" s="9"/>
@@ -6601,7 +6613,7 @@
       <c r="F11" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G11" s="32">
+      <c r="G11" s="27">
         <v>46325</v>
       </c>
       <c r="H11" s="9"/>
@@ -6625,7 +6637,7 @@
       <c r="F12" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="32">
+      <c r="G12" s="27">
         <v>46326</v>
       </c>
       <c r="H12" s="9"/>
@@ -6649,11 +6661,11 @@
       <c r="F13" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="27">
         <v>46327</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
@@ -6675,7 +6687,7 @@
       <c r="F14" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="27">
         <v>46328</v>
       </c>
       <c r="H14" s="9"/>
@@ -6699,7 +6711,7 @@
       <c r="F15" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="32">
+      <c r="G15" s="27">
         <v>46329</v>
       </c>
       <c r="H15" s="9"/>
@@ -6723,7 +6735,7 @@
       <c r="F16" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G16" s="32">
+      <c r="G16" s="27">
         <v>46330</v>
       </c>
       <c r="H16" s="9"/>
@@ -6747,7 +6759,7 @@
       <c r="F17" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G17" s="32">
+      <c r="G17" s="27">
         <v>46331</v>
       </c>
       <c r="H17" s="9"/>
@@ -6771,7 +6783,7 @@
       <c r="F18" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G18" s="32">
+      <c r="G18" s="27">
         <v>46332</v>
       </c>
       <c r="H18" s="9"/>
@@ -6795,23 +6807,23 @@
       <c r="F19" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G19" s="32">
+      <c r="G19" s="27">
         <v>46333</v>
       </c>
       <c r="H19" s="9"/>
     </row>
     <row r="20" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="C20" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>182</v>
-      </c>
       <c r="D20" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>112</v>
@@ -6819,23 +6831,23 @@
       <c r="F20" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G20" s="32">
+      <c r="G20" s="27">
         <v>46334</v>
       </c>
       <c r="H20" s="9"/>
     </row>
     <row r="21" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="C21" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="D21" s="9" t="s">
         <v>188</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>189</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>112</v>
@@ -6843,23 +6855,23 @@
       <c r="F21" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G21" s="32">
+      <c r="G21" s="27">
         <v>46335</v>
       </c>
       <c r="H21" s="9"/>
     </row>
     <row r="22" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="D22" s="9" t="s">
         <v>195</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>196</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>112</v>
@@ -6867,23 +6879,23 @@
       <c r="F22" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G22" s="32">
+      <c r="G22" s="27">
         <v>46336</v>
       </c>
       <c r="H22" s="9"/>
     </row>
     <row r="23" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="C23" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>200</v>
-      </c>
       <c r="D23" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>112</v>
@@ -6891,23 +6903,23 @@
       <c r="F23" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G23" s="32">
+      <c r="G23" s="27">
         <v>46337</v>
       </c>
       <c r="H23" s="9"/>
     </row>
     <row r="24" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B24" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="B24" s="9" t="s">
-        <v>211</v>
-      </c>
       <c r="C24" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>214</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>112</v>
@@ -6915,23 +6927,23 @@
       <c r="F24" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G24" s="32">
+      <c r="G24" s="27">
         <v>46338</v>
       </c>
       <c r="H24" s="9"/>
     </row>
     <row r="25" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="B25" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>216</v>
-      </c>
       <c r="C25" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>218</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>219</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>112</v>
@@ -6939,23 +6951,23 @@
       <c r="F25" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G25" s="32">
+      <c r="G25" s="27">
         <v>46339</v>
       </c>
       <c r="H25" s="9"/>
     </row>
     <row r="26" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="C26" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="C26" s="9" t="s">
-        <v>223</v>
-      </c>
       <c r="D26" s="9" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>112</v>
@@ -6963,23 +6975,23 @@
       <c r="F26" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G26" s="32">
+      <c r="G26" s="27">
         <v>46340</v>
       </c>
       <c r="H26" s="9"/>
     </row>
     <row r="27" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B27" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="D27" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>112</v>
@@ -6987,23 +6999,23 @@
       <c r="F27" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G27" s="32">
+      <c r="G27" s="27">
         <v>46341</v>
       </c>
       <c r="H27" s="9"/>
     </row>
     <row r="28" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C28" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>236</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>237</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>112</v>
@@ -7011,23 +7023,23 @@
       <c r="F28" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G28" s="32">
+      <c r="G28" s="27">
         <v>46342</v>
       </c>
       <c r="H28" s="9"/>
     </row>
     <row r="29" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>89</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>112</v>
@@ -7035,23 +7047,23 @@
       <c r="F29" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G29" s="32">
+      <c r="G29" s="27">
         <v>46343</v>
       </c>
       <c r="H29" s="9"/>
     </row>
     <row r="30" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="B30" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="B30" s="9" t="s">
-        <v>244</v>
-      </c>
       <c r="C30" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>246</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>247</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>112</v>
@@ -7059,25 +7071,25 @@
       <c r="F30" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G30" s="32">
+      <c r="G30" s="27">
         <v>46344</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B31" s="9" t="s">
         <v>91</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="D31" s="9" t="s">
         <v>251</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>252</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>112</v>
@@ -7085,23 +7097,23 @@
       <c r="F31" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G31" s="32">
+      <c r="G31" s="27">
         <v>46345</v>
       </c>
       <c r="H31" s="9"/>
     </row>
     <row r="32" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>92</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>256</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>257</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>112</v>
@@ -7109,71 +7121,75 @@
       <c r="F32" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G32" s="32">
+      <c r="G32" s="27">
         <v>46346</v>
       </c>
       <c r="H32" s="9"/>
     </row>
-    <row r="33" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B33" s="9" t="s">
         <v>94</v>
       </c>
       <c r="C33" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="D33" s="9" t="s">
         <v>260</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>261</v>
       </c>
       <c r="E33" s="8" t="s">
         <v>112</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="G33" s="32">
+        <v>63</v>
+      </c>
+      <c r="G33" s="27">
         <v>46347</v>
       </c>
-      <c r="H33" s="9"/>
-    </row>
-    <row r="34" spans="1:8" ht="69" x14ac:dyDescent="0.3">
+      <c r="H33" s="9" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B34" s="9" t="s">
         <v>95</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="D34" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>266</v>
-      </c>
       <c r="E34" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="G34" s="32">
+        <v>63</v>
+      </c>
+      <c r="G34" s="27">
         <v>46348</v>
       </c>
-      <c r="H34" s="9"/>
+      <c r="H34" s="9" t="s">
+        <v>473</v>
+      </c>
     </row>
     <row r="35" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B35" s="9" t="s">
         <v>96</v>
       </c>
       <c r="C35" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="D35" s="9" t="s">
         <v>270</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>271</v>
       </c>
       <c r="E35" s="8" t="s">
         <v>112</v>
@@ -7181,23 +7197,23 @@
       <c r="F35" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G35" s="32">
+      <c r="G35" s="27">
         <v>46349</v>
       </c>
       <c r="H35" s="9"/>
     </row>
     <row r="36" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>98</v>
       </c>
       <c r="C36" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="D36" s="9" t="s">
         <v>274</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>275</v>
       </c>
       <c r="E36" s="8" t="s">
         <v>112</v>
@@ -7205,267 +7221,267 @@
       <c r="F36" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G36" s="32">
+      <c r="G36" s="27">
         <v>46350</v>
       </c>
       <c r="H36" s="9"/>
     </row>
     <row r="37" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B37" s="9" t="s">
         <v>99</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G37" s="32">
+      <c r="G37" s="27">
         <v>46351</v>
       </c>
       <c r="H37" s="9"/>
     </row>
     <row r="38" spans="1:8" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B38" s="9" t="s">
         <v>101</v>
       </c>
       <c r="C38" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="D38" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="D38" s="9" t="s">
-        <v>289</v>
-      </c>
       <c r="E38" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F38" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G38" s="32">
+      <c r="G38" s="27">
         <v>46352</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B39" s="9" t="s">
         <v>104</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G39" s="32">
+      <c r="G39" s="27">
         <v>46353</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B40" s="9" t="s">
         <v>109</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F40" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G40" s="32">
+      <c r="G40" s="27">
         <v>46354</v>
       </c>
       <c r="H40" s="9"/>
     </row>
     <row r="41" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>113</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F41" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G41" s="32">
+      <c r="G41" s="27">
         <v>46355</v>
       </c>
       <c r="H41" s="9"/>
     </row>
     <row r="42" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B42" s="9" t="s">
         <v>115</v>
       </c>
       <c r="C42" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="D42" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>320</v>
-      </c>
       <c r="E42" s="8" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F42" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G42" s="32">
+      <c r="G42" s="27">
         <v>46356</v>
       </c>
       <c r="H42" s="9"/>
     </row>
     <row r="43" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B43" s="9" t="s">
         <v>118</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F43" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G43" s="32">
+      <c r="G43" s="27">
         <v>46357</v>
       </c>
       <c r="H43" s="9"/>
     </row>
     <row r="44" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B44" s="9" t="s">
         <v>122</v>
       </c>
       <c r="C44" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="D44" s="9" t="s">
         <v>336</v>
       </c>
-      <c r="D44" s="9" t="s">
-        <v>338</v>
-      </c>
       <c r="E44" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F44" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G44" s="32">
+      <c r="G44" s="27">
         <v>46358</v>
       </c>
       <c r="H44" s="9"/>
     </row>
     <row r="45" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B45" s="9" t="s">
         <v>125</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G45" s="32">
+      <c r="G45" s="27">
         <v>46359</v>
       </c>
       <c r="H45" s="9"/>
     </row>
     <row r="46" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B46" s="9" t="s">
         <v>127</v>
       </c>
       <c r="C46" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="D46" s="9" t="s">
         <v>354</v>
       </c>
-      <c r="D46" s="9" t="s">
-        <v>356</v>
-      </c>
       <c r="E46" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F46" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G46" s="32">
+      <c r="G46" s="27">
         <v>46360</v>
       </c>
       <c r="H46" s="9"/>
     </row>
     <row r="47" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B47" s="9" t="s">
         <v>132</v>
       </c>
       <c r="C47" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="D47" s="9" t="s">
         <v>364</v>
-      </c>
-      <c r="D47" s="9" t="s">
-        <v>366</v>
       </c>
       <c r="E47" s="8" t="s">
         <v>112</v>
@@ -7473,23 +7489,23 @@
       <c r="F47" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G47" s="32">
+      <c r="G47" s="27">
         <v>46361</v>
       </c>
       <c r="H47" s="9"/>
     </row>
     <row r="48" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>133</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="E48" s="8" t="s">
         <v>112</v>
@@ -7497,23 +7513,23 @@
       <c r="F48" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G48" s="32">
+      <c r="G48" s="27">
         <v>46362</v>
       </c>
       <c r="H48" s="9"/>
     </row>
     <row r="49" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A49" s="8" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B49" s="9" t="s">
         <v>135</v>
       </c>
       <c r="C49" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="D49" s="9" t="s">
         <v>382</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>384</v>
       </c>
       <c r="E49" s="8" t="s">
         <v>112</v>
@@ -7521,23 +7537,23 @@
       <c r="F49" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G49" s="32">
+      <c r="G49" s="27">
         <v>46363</v>
       </c>
       <c r="H49" s="9"/>
     </row>
     <row r="50" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B50" s="9" t="s">
         <v>139</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>112</v>
@@ -7545,61 +7561,61 @@
       <c r="F50" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G50" s="32">
+      <c r="G50" s="27">
         <v>46364</v>
       </c>
       <c r="H50" s="9"/>
     </row>
     <row r="51" spans="1:8" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B51" s="9" t="s">
         <v>145</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F51" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G51" s="32">
+      <c r="G51" s="27">
         <v>46365</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="165.6" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B52" s="9" t="s">
         <v>148</v>
       </c>
       <c r="C52" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="D52" s="9" t="s">
         <v>400</v>
       </c>
-      <c r="D52" s="9" t="s">
-        <v>402</v>
-      </c>
       <c r="E52" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F52" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G52" s="32">
+      <c r="G52" s="27">
         <v>46366</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>
@@ -7670,15 +7686,15 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="16">
         <f>COUNTIF(F9:F28, "Passed")</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="B6" s="17">
         <f>COUNTIF(F9:F28, "Failed")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C6" s="18">
         <f>COUNTBLANK(F9:F28) + COUNTIF(F9:F28, "Untested")</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D6" s="19">
         <f>COUNTIF(F9:F28, "Blocked")</f>
@@ -7721,402 +7737,486 @@
     </row>
     <row r="9" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>285</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
+      <c r="F9" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="27">
+        <v>46323</v>
+      </c>
       <c r="H9" s="9"/>
     </row>
     <row r="10" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>158</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="27">
+        <v>46323</v>
+      </c>
       <c r="H10" s="9"/>
     </row>
     <row r="11" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>170</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="27">
+        <v>46323</v>
+      </c>
       <c r="H11" s="9"/>
     </row>
     <row r="12" spans="1:8" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>174</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="27">
+        <v>46323</v>
+      </c>
       <c r="H12" s="9"/>
     </row>
     <row r="13" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>179</v>
+        <v>469</v>
       </c>
       <c r="C13" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>319</v>
       </c>
-      <c r="D13" s="9" t="s">
-        <v>321</v>
-      </c>
       <c r="E13" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G13" s="27">
+        <v>46323</v>
+      </c>
       <c r="H13" s="9"/>
     </row>
     <row r="14" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>137</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" s="27">
+        <v>46323</v>
+      </c>
       <c r="H14" s="9"/>
     </row>
     <row r="15" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>143</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="9"/>
+        <v>276</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="27">
+        <v>46323</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>474</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>149</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G16" s="27">
+        <v>46323</v>
+      </c>
       <c r="H16" s="9"/>
     </row>
     <row r="17" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>154</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G17" s="27">
+        <v>46323</v>
+      </c>
       <c r="H17" s="9"/>
     </row>
     <row r="18" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G18" s="27">
+        <v>46323</v>
+      </c>
       <c r="H18" s="9"/>
     </row>
     <row r="19" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C19" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>365</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>367</v>
-      </c>
       <c r="E19" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G19" s="27">
+        <v>46323</v>
+      </c>
       <c r="H19" s="9"/>
     </row>
     <row r="20" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
+        <v>359</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G20" s="27">
+        <v>46323</v>
+      </c>
       <c r="H20" s="9"/>
     </row>
     <row r="21" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>383</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>385</v>
-      </c>
       <c r="E21" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
+        <v>359</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G21" s="27">
+        <v>46323</v>
+      </c>
       <c r="H21" s="9"/>
     </row>
     <row r="22" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>369</v>
-      </c>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
+        <v>367</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G22" s="27">
+        <v>46323</v>
+      </c>
       <c r="H22" s="9"/>
     </row>
     <row r="23" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C23" s="9" t="s">
+        <v>394</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>396</v>
       </c>
-      <c r="D23" s="9" t="s">
-        <v>398</v>
-      </c>
       <c r="E23" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+        <v>359</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G23" s="27">
+        <v>46323</v>
+      </c>
       <c r="H23" s="9"/>
     </row>
     <row r="24" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="9"/>
+        <v>359</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="G24" s="27">
+        <v>46323</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>474</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>406</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>408</v>
-      </c>
       <c r="E25" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
+        <v>359</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G25" s="27">
+        <v>46323</v>
+      </c>
       <c r="H25" s="9"/>
     </row>
     <row r="26" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>409</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>411</v>
-      </c>
       <c r="D26" s="9" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
+        <v>359</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G26" s="27">
+        <v>46323</v>
+      </c>
       <c r="H26" s="9"/>
     </row>
     <row r="27" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
+        <v>413</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>415</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>417</v>
-      </c>
       <c r="D27" s="9" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
+        <v>276</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G27" s="27">
+        <v>46323</v>
+      </c>
       <c r="H27" s="9"/>
     </row>
     <row r="28" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>420</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>422</v>
-      </c>
       <c r="D28" s="9" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
+        <v>359</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G28" s="27">
+        <v>46323</v>
+      </c>
       <c r="H28" s="9"/>
     </row>
   </sheetData>
@@ -8146,7 +8246,7 @@
         <v>44</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G2" s="21" t="s">
         <v>4</v>
@@ -8157,7 +8257,7 @@
         <v>53</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -8242,16 +8342,16 @@
     </row>
     <row r="9" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>325</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>327</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>329</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>119</v>
@@ -8262,19 +8362,19 @@
     </row>
     <row r="10" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
@@ -8282,19 +8382,19 @@
     </row>
     <row r="11" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>342</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="C11" s="9" t="s">
+      <c r="D11" s="9" t="s">
         <v>344</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>346</v>
-      </c>
       <c r="E11" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
@@ -8302,19 +8402,19 @@
     </row>
     <row r="12" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
@@ -8322,19 +8422,19 @@
     </row>
     <row r="13" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -8342,19 +8442,19 @@
     </row>
     <row r="14" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
@@ -8362,19 +8462,19 @@
     </row>
     <row r="15" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
@@ -8382,19 +8482,19 @@
     </row>
     <row r="16" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -8402,19 +8502,19 @@
     </row>
     <row r="17" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
@@ -8422,19 +8522,19 @@
     </row>
     <row r="18" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>419</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>421</v>
-      </c>
       <c r="E18" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
@@ -8442,19 +8542,19 @@
     </row>
     <row r="19" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>424</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>425</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>426</v>
-      </c>
       <c r="E19" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
@@ -8462,19 +8562,19 @@
     </row>
     <row r="20" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
+        <v>425</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>427</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>428</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>429</v>
-      </c>
       <c r="E20" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
@@ -8482,19 +8582,19 @@
     </row>
     <row r="21" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
+        <v>428</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>430</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>279</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>431</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>432</v>
-      </c>
       <c r="E21" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
@@ -8502,19 +8602,19 @@
     </row>
     <row r="22" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
+        <v>431</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>433</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>434</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>435</v>
-      </c>
       <c r="E22" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
@@ -8522,19 +8622,19 @@
     </row>
     <row r="23" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>436</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>287</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>437</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>438</v>
-      </c>
       <c r="E23" s="8" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
@@ -8542,19 +8642,19 @@
     </row>
     <row r="24" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>439</v>
       </c>
-      <c r="B24" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>440</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>441</v>
-      </c>
       <c r="E24" s="8" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
@@ -8562,19 +8662,19 @@
     </row>
     <row r="25" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
+        <v>440</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>442</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>298</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>443</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>444</v>
-      </c>
       <c r="E25" s="8" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
@@ -8582,19 +8682,19 @@
     </row>
     <row r="26" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
+        <v>443</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>445</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>446</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>447</v>
-      </c>
       <c r="E26" s="8" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
@@ -8602,19 +8702,19 @@
     </row>
     <row r="27" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
+        <v>446</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>448</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>317</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>449</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>450</v>
-      </c>
       <c r="E27" s="8" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
@@ -8622,19 +8722,19 @@
     </row>
     <row r="28" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
+        <v>449</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>451</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>326</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>452</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>453</v>
-      </c>
       <c r="E28" s="8" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
@@ -8660,16 +8760,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B2" s="27" t="s">
-        <v>454</v>
-      </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
+      <c r="B2" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
     </row>
     <row r="4" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
@@ -8704,7 +8804,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>12</v>
@@ -8715,10 +8815,10 @@
     </row>
     <row r="7" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>16</v>
@@ -8732,13 +8832,13 @@
         <v>27</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>458</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>460</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>62</v>
@@ -8750,7 +8850,7 @@
         <v>65</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
@@ -8762,7 +8862,7 @@
       </c>
       <c r="D11" s="8">
         <f>'Admin - Orders'!A6</f>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E11" s="8">
         <f>'Admin - Orders'!B6</f>
@@ -8774,7 +8874,7 @@
       </c>
       <c r="G11" s="8">
         <f>'Admin - Orders'!D6</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H11" s="8">
         <f>'Admin - Orders'!E6</f>
@@ -8794,15 +8894,15 @@
       </c>
       <c r="D12" s="8">
         <f>'Admin - Shipments'!A6</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E12" s="8">
         <f>'Admin - Shipments'!B6</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" s="8">
         <f>'Admin - Shipments'!C6</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G12" s="8">
         <f>'Admin - Shipments'!D6</f>
@@ -8822,7 +8922,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D13" s="8">
         <f>'Admin - Gift cards'!A6</f>
@@ -8851,23 +8951,23 @@
     </row>
     <row r="14" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C14" s="24" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D14" s="13">
         <f t="shared" ref="D14:I14" si="0">SUM(D11:D13)</f>
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="E14" s="13">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F14" s="13">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G14" s="13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H14" s="13">
         <f t="shared" si="0"/>
@@ -8880,26 +8980,26 @@
     </row>
     <row r="16" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C16" s="25" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="E16" s="26">
         <f>IF(I14-H14=0, 0, (D14+E14)/(I14-H14)*100)</f>
-        <v>52.380952380952387</v>
+        <v>73.80952380952381</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="17" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C17" s="25" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="E17" s="26">
         <f>IF(D14+E14=0, 0, D14/(D14+E14)*100)</f>
-        <v>88.63636363636364</v>
+        <v>88.709677419354833</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="21" spans="3:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Thực hiện automation testing của modul quản lý thẻ quà tặng admin_giftcard
</commit_message>
<xml_diff>
--- a/23130064_TruongCaoDoan/Group13_23130064_TruongCaoDoan.xlsx
+++ b/23130064_TruongCaoDoan/Group13_23130064_TruongCaoDoan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\n4k1\test\gh\Tester\23130064_TruongCaoDoan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B7327B-A903-47F7-9CE7-67A727CB3690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF982EC-322E-4881-A4BB-0A39AF01F5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="477">
   <si>
     <t>TEST CASE SPECIFICATION</t>
   </si>
@@ -144,9 +144,6 @@
     <t>Pre-Condition</t>
   </si>
   <si>
-    <t>Bắt đầu tài liệu, thiết kế Test Design, test case cho chức năng (quản lý đơn hàng, quản lý giao hàng và quản lý gift card)</t>
-  </si>
-  <si>
     <t>Quản lý Đơn hàng (Orders)</t>
   </si>
   <si>
@@ -920,9 +917,6 @@
   </si>
   <si>
     <t>1. Số lượng dòng dữ liệu hiển thị trên bảng cập nhật tương ứng chính xác theo giá trị đã chọn.</t>
-  </si>
-  <si>
-    <t>Ràng buộc dữ liệu</t>
   </si>
   <si>
     <t>admin_ord_28</t>
@@ -1690,6 +1684,21 @@
   </si>
   <si>
     <t>Thực tế hệ thống tiến hành tìm kiếm chứ không thông báo ngày nhận không hợp lệ</t>
+  </si>
+  <si>
+    <t>Thực tế hệ thống không thông báo "giá trị thẻ quà tặng phải lớn hơn 0" 
+Hệ thống lưu thẻ quà tặng</t>
+  </si>
+  <si>
+    <t>Thực tế hệ thống không thông báo "buộc nhập tên người nhận" 
+Hệ thống lưu thẻ quà tặng</t>
+  </si>
+  <si>
+    <t>Thực tế hệ thống không thông báo "bắt buộc nhập email người nhận đối với thẻ ảo" 
+Hệ thống lưu thẻ quà tặng</t>
+  </si>
+  <si>
+    <t>Thực hiện automatio danh sách test case của module quản lý thẻ quà tặng  admin_giftcard</t>
   </si>
 </sst>
 </file>
@@ -1887,7 +1896,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1967,6 +1976,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2286,19 +2301,19 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="69" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" ht="55.2" x14ac:dyDescent="0.3">
       <c r="B12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>17</v>
+      <c r="C12" s="8">
+        <v>1.2</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="8" t="s">
         <v>31</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>33</v>
+        <v>476</v>
       </c>
       <c r="G12" s="9"/>
     </row>
@@ -3360,16 +3375,16 @@
         <v>1</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E9" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>38</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="41.4" x14ac:dyDescent="0.3">
@@ -3377,16 +3392,16 @@
         <v>2</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
@@ -3394,16 +3409,16 @@
         <v>3</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -4411,39 +4426,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>57</v>
-      </c>
       <c r="D2" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="14" t="s">
         <v>59</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>60</v>
       </c>
       <c r="F2" s="9"/>
     </row>
@@ -4452,10 +4467,10 @@
       <c r="B3" s="9"/>
       <c r="C3" s="31"/>
       <c r="D3" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F3" s="9"/>
     </row>
@@ -4464,10 +4479,10 @@
       <c r="B4" s="9"/>
       <c r="C4" s="32"/>
       <c r="D4" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F4" s="9"/>
     </row>
@@ -4475,13 +4490,13 @@
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="15" t="s">
         <v>69</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>70</v>
       </c>
       <c r="F5" s="9"/>
     </row>
@@ -4490,10 +4505,10 @@
       <c r="B6" s="9"/>
       <c r="C6" s="31"/>
       <c r="D6" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F6" s="9"/>
     </row>
@@ -4502,10 +4517,10 @@
       <c r="B7" s="9"/>
       <c r="C7" s="31"/>
       <c r="D7" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F7" s="9"/>
     </row>
@@ -4514,10 +4529,10 @@
       <c r="B8" s="9"/>
       <c r="C8" s="32"/>
       <c r="D8" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F8" s="9"/>
     </row>
@@ -4525,13 +4540,13 @@
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="30" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>75</v>
-      </c>
       <c r="E9" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F9" s="9"/>
     </row>
@@ -4540,10 +4555,10 @@
       <c r="B10" s="9"/>
       <c r="C10" s="31"/>
       <c r="D10" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F10" s="9"/>
     </row>
@@ -4552,10 +4567,10 @@
       <c r="B11" s="9"/>
       <c r="C11" s="31"/>
       <c r="D11" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F11" s="9"/>
     </row>
@@ -4564,10 +4579,10 @@
       <c r="B12" s="9"/>
       <c r="C12" s="31"/>
       <c r="D12" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F12" s="9"/>
     </row>
@@ -4576,10 +4591,10 @@
       <c r="B13" s="9"/>
       <c r="C13" s="31"/>
       <c r="D13" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F13" s="9"/>
     </row>
@@ -4588,10 +4603,10 @@
       <c r="B14" s="9"/>
       <c r="C14" s="31"/>
       <c r="D14" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F14" s="9"/>
     </row>
@@ -4600,10 +4615,10 @@
       <c r="B15" s="9"/>
       <c r="C15" s="31"/>
       <c r="D15" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F15" s="9"/>
     </row>
@@ -4612,10 +4627,10 @@
       <c r="B16" s="9"/>
       <c r="C16" s="31"/>
       <c r="D16" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F16" s="9"/>
     </row>
@@ -4624,10 +4639,10 @@
       <c r="B17" s="9"/>
       <c r="C17" s="31"/>
       <c r="D17" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F17" s="9"/>
     </row>
@@ -4636,10 +4651,10 @@
       <c r="B18" s="9"/>
       <c r="C18" s="31"/>
       <c r="D18" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F18" s="9"/>
     </row>
@@ -4648,10 +4663,10 @@
       <c r="B19" s="9"/>
       <c r="C19" s="31"/>
       <c r="D19" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F19" s="9"/>
     </row>
@@ -4660,10 +4675,10 @@
       <c r="B20" s="9"/>
       <c r="C20" s="31"/>
       <c r="D20" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F20" s="9"/>
     </row>
@@ -4672,10 +4687,10 @@
       <c r="B21" s="9"/>
       <c r="C21" s="32"/>
       <c r="D21" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F21" s="9"/>
     </row>
@@ -4683,13 +4698,13 @@
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>89</v>
-      </c>
       <c r="E22" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F22" s="9"/>
     </row>
@@ -4698,10 +4713,10 @@
       <c r="B23" s="9"/>
       <c r="C23" s="31"/>
       <c r="D23" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F23" s="9"/>
     </row>
@@ -4710,10 +4725,10 @@
       <c r="B24" s="9"/>
       <c r="C24" s="31"/>
       <c r="D24" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F24" s="9"/>
     </row>
@@ -4722,10 +4737,10 @@
       <c r="B25" s="9"/>
       <c r="C25" s="32"/>
       <c r="D25" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F25" s="9"/>
     </row>
@@ -4733,13 +4748,13 @@
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="D26" s="9" t="s">
-        <v>94</v>
-      </c>
       <c r="E26" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F26" s="9"/>
     </row>
@@ -4748,10 +4763,10 @@
       <c r="B27" s="9"/>
       <c r="C27" s="31"/>
       <c r="D27" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F27" s="9"/>
     </row>
@@ -4760,10 +4775,10 @@
       <c r="B28" s="9"/>
       <c r="C28" s="32"/>
       <c r="D28" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F28" s="9"/>
     </row>
@@ -4771,13 +4786,13 @@
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
       <c r="C29" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="D29" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="D29" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="E29" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F29" s="9"/>
     </row>
@@ -4786,10 +4801,10 @@
       <c r="B30" s="9"/>
       <c r="C30" s="32"/>
       <c r="D30" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F30" s="9"/>
     </row>
@@ -4797,13 +4812,13 @@
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>101</v>
-      </c>
       <c r="E31" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F31" s="9"/>
     </row>
@@ -4812,10 +4827,10 @@
       <c r="B32" s="9"/>
       <c r="C32" s="31"/>
       <c r="D32" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F32" s="9"/>
     </row>
@@ -4824,10 +4839,10 @@
       <c r="B33" s="9"/>
       <c r="C33" s="32"/>
       <c r="D33" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F33" s="9"/>
     </row>
@@ -4835,13 +4850,13 @@
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="30" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F34" s="9"/>
     </row>
@@ -4850,10 +4865,10 @@
       <c r="B35" s="9"/>
       <c r="C35" s="31"/>
       <c r="D35" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F35" s="9"/>
     </row>
@@ -4862,10 +4877,10 @@
       <c r="B36" s="9"/>
       <c r="C36" s="32"/>
       <c r="D36" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F36" s="9"/>
     </row>
@@ -4873,13 +4888,13 @@
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F37" s="9"/>
     </row>
@@ -4888,10 +4903,10 @@
       <c r="B38" s="9"/>
       <c r="C38" s="31"/>
       <c r="D38" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F38" s="9"/>
     </row>
@@ -4900,10 +4915,10 @@
       <c r="B39" s="9"/>
       <c r="C39" s="32"/>
       <c r="D39" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E39" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F39" s="9"/>
     </row>
@@ -4911,13 +4926,13 @@
       <c r="A40" s="9"/>
       <c r="B40" s="9"/>
       <c r="C40" s="30" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F40" s="9"/>
     </row>
@@ -4926,10 +4941,10 @@
       <c r="B41" s="9"/>
       <c r="C41" s="31"/>
       <c r="D41" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E41" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F41" s="9"/>
     </row>
@@ -4938,10 +4953,10 @@
       <c r="B42" s="9"/>
       <c r="C42" s="31"/>
       <c r="D42" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F42" s="9"/>
     </row>
@@ -4950,10 +4965,10 @@
       <c r="B43" s="9"/>
       <c r="C43" s="32"/>
       <c r="D43" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F43" s="9"/>
     </row>
@@ -4961,13 +4976,13 @@
       <c r="A44" s="9"/>
       <c r="B44" s="9"/>
       <c r="C44" s="30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F44" s="9"/>
     </row>
@@ -4976,26 +4991,26 @@
       <c r="B45" s="9"/>
       <c r="C45" s="32"/>
       <c r="D45" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F45" s="9"/>
     </row>
     <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A46" s="9"/>
       <c r="B46" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C46" s="30" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F46" s="9"/>
     </row>
@@ -5004,10 +5019,10 @@
       <c r="B47" s="9"/>
       <c r="C47" s="32"/>
       <c r="D47" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F47" s="9"/>
     </row>
@@ -5015,13 +5030,13 @@
       <c r="A48" s="9"/>
       <c r="B48" s="9"/>
       <c r="C48" s="30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F48" s="9"/>
     </row>
@@ -5030,10 +5045,10 @@
       <c r="B49" s="9"/>
       <c r="C49" s="31"/>
       <c r="D49" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E49" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F49" s="9"/>
     </row>
@@ -5042,10 +5057,10 @@
       <c r="B50" s="9"/>
       <c r="C50" s="31"/>
       <c r="D50" s="9" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F50" s="9"/>
     </row>
@@ -5054,10 +5069,10 @@
       <c r="B51" s="9"/>
       <c r="C51" s="31"/>
       <c r="D51" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E51" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F51" s="9"/>
     </row>
@@ -5066,10 +5081,10 @@
       <c r="B52" s="9"/>
       <c r="C52" s="31"/>
       <c r="D52" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F52" s="9"/>
     </row>
@@ -5078,10 +5093,10 @@
       <c r="B53" s="9"/>
       <c r="C53" s="31"/>
       <c r="D53" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E53" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F53" s="9"/>
     </row>
@@ -5090,10 +5105,10 @@
       <c r="B54" s="9"/>
       <c r="C54" s="32"/>
       <c r="D54" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F54" s="9"/>
     </row>
@@ -5101,13 +5116,13 @@
       <c r="A55" s="9"/>
       <c r="B55" s="9"/>
       <c r="C55" s="30" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F55" s="9"/>
     </row>
@@ -5116,10 +5131,10 @@
       <c r="B56" s="9"/>
       <c r="C56" s="32"/>
       <c r="D56" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F56" s="9"/>
     </row>
@@ -5127,13 +5142,13 @@
       <c r="A57" s="9"/>
       <c r="B57" s="9"/>
       <c r="C57" s="30" t="s">
+        <v>203</v>
+      </c>
+      <c r="D57" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="D57" s="9" t="s">
-        <v>205</v>
-      </c>
       <c r="E57" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F57" s="9"/>
     </row>
@@ -5142,10 +5157,10 @@
       <c r="B58" s="9"/>
       <c r="C58" s="31"/>
       <c r="D58" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F58" s="9"/>
     </row>
@@ -5154,10 +5169,10 @@
       <c r="B59" s="9"/>
       <c r="C59" s="31"/>
       <c r="D59" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E59" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F59" s="9"/>
     </row>
@@ -5166,10 +5181,10 @@
       <c r="B60" s="9"/>
       <c r="C60" s="31"/>
       <c r="D60" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E60" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F60" s="9"/>
     </row>
@@ -5178,10 +5193,10 @@
       <c r="B61" s="9"/>
       <c r="C61" s="31"/>
       <c r="D61" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E61" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F61" s="9"/>
     </row>
@@ -5190,10 +5205,10 @@
       <c r="B62" s="9"/>
       <c r="C62" s="32"/>
       <c r="D62" s="9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E62" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F62" s="9"/>
     </row>
@@ -5201,13 +5216,13 @@
       <c r="A63" s="9"/>
       <c r="B63" s="9"/>
       <c r="C63" s="30" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E63" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F63" s="9"/>
     </row>
@@ -5216,10 +5231,10 @@
       <c r="B64" s="9"/>
       <c r="C64" s="31"/>
       <c r="D64" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E64" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F64" s="9"/>
     </row>
@@ -5228,26 +5243,26 @@
       <c r="B65" s="9"/>
       <c r="C65" s="32"/>
       <c r="D65" s="9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E65" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F65" s="9"/>
     </row>
     <row r="66" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A66" s="9"/>
       <c r="B66" s="11" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C66" s="30" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E66" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F66" s="9"/>
     </row>
@@ -5256,10 +5271,10 @@
       <c r="B67" s="9"/>
       <c r="C67" s="31"/>
       <c r="D67" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E67" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F67" s="9"/>
     </row>
@@ -5268,10 +5283,10 @@
       <c r="B68" s="9"/>
       <c r="C68" s="31"/>
       <c r="D68" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E68" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F68" s="9"/>
     </row>
@@ -5280,10 +5295,10 @@
       <c r="B69" s="9"/>
       <c r="C69" s="31"/>
       <c r="D69" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E69" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F69" s="9"/>
     </row>
@@ -5292,10 +5307,10 @@
       <c r="B70" s="9"/>
       <c r="C70" s="31"/>
       <c r="D70" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E70" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F70" s="9"/>
     </row>
@@ -5304,10 +5319,10 @@
       <c r="B71" s="9"/>
       <c r="C71" s="32"/>
       <c r="D71" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E71" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F71" s="9"/>
     </row>
@@ -5315,111 +5330,109 @@
       <c r="A72" s="9"/>
       <c r="B72" s="9"/>
       <c r="C72" s="30" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E72" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F72" s="9"/>
     </row>
     <row r="73" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A73" s="9"/>
       <c r="B73" s="9"/>
-      <c r="C73" s="31"/>
+      <c r="C73" s="33"/>
       <c r="D73" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E73" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F73" s="9"/>
     </row>
     <row r="74" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A74" s="9"/>
       <c r="B74" s="9"/>
-      <c r="C74" s="31"/>
+      <c r="C74" s="33"/>
       <c r="D74" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E74" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F74" s="9"/>
     </row>
     <row r="75" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A75" s="9"/>
       <c r="B75" s="9"/>
-      <c r="C75" s="31"/>
+      <c r="C75" s="33"/>
       <c r="D75" s="9" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E75" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F75" s="9"/>
     </row>
     <row r="76" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A76" s="9"/>
       <c r="B76" s="9"/>
-      <c r="C76" s="32"/>
+      <c r="C76" s="33"/>
       <c r="D76" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E76" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F76" s="9"/>
     </row>
     <row r="77" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A77" s="9"/>
       <c r="B77" s="9"/>
-      <c r="C77" s="30" t="s">
-        <v>271</v>
-      </c>
+      <c r="C77" s="33"/>
       <c r="D77" s="9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="E77" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F77" s="9"/>
     </row>
     <row r="78" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A78" s="9"/>
       <c r="B78" s="9"/>
-      <c r="C78" s="31"/>
+      <c r="C78" s="33"/>
       <c r="D78" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E78" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F78" s="9"/>
     </row>
     <row r="79" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A79" s="9"/>
       <c r="B79" s="9"/>
-      <c r="C79" s="31"/>
+      <c r="C79" s="33"/>
       <c r="D79" s="9" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E79" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F79" s="9"/>
     </row>
     <row r="80" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A80" s="9"/>
       <c r="B80" s="9"/>
-      <c r="C80" s="32"/>
+      <c r="C80" s="34"/>
       <c r="D80" s="9" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E80" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F80" s="9"/>
     </row>
@@ -5427,13 +5440,13 @@
       <c r="A81" s="9"/>
       <c r="B81" s="9"/>
       <c r="C81" s="30" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="E81" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F81" s="9"/>
     </row>
@@ -5442,10 +5455,10 @@
       <c r="B82" s="9"/>
       <c r="C82" s="32"/>
       <c r="D82" s="9" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E82" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F82" s="9"/>
     </row>
@@ -5453,13 +5466,13 @@
       <c r="A83" s="9"/>
       <c r="B83" s="9"/>
       <c r="C83" s="12" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F83" s="9"/>
     </row>
@@ -5467,13 +5480,13 @@
       <c r="A84" s="9"/>
       <c r="B84" s="9"/>
       <c r="C84" s="22" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E84" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F84" s="9"/>
     </row>
@@ -5481,13 +5494,13 @@
       <c r="A85" s="9"/>
       <c r="B85" s="9"/>
       <c r="C85" s="23" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D85" s="9" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E85" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F85" s="9"/>
     </row>
@@ -6407,19 +6420,7 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="C5:C8"/>
-    <mergeCell ref="C9:C21"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="C57:C62"/>
-    <mergeCell ref="C63:C65"/>
-    <mergeCell ref="C66:C71"/>
-    <mergeCell ref="C72:C76"/>
-    <mergeCell ref="C77:C80"/>
+  <mergeCells count="19">
     <mergeCell ref="C81:C82"/>
     <mergeCell ref="C34:C36"/>
     <mergeCell ref="C37:C39"/>
@@ -6428,6 +6429,17 @@
     <mergeCell ref="C46:C47"/>
     <mergeCell ref="C48:C54"/>
     <mergeCell ref="C55:C56"/>
+    <mergeCell ref="C72:C80"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="C57:C62"/>
+    <mergeCell ref="C63:C65"/>
+    <mergeCell ref="C66:C71"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="C9:C21"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="C26:C28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -6452,23 +6464,23 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
@@ -6476,22 +6488,22 @@
     </row>
     <row r="5" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="13" t="s">
-        <v>63</v>
-      </c>
       <c r="E5" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>65</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -6522,48 +6534,48 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>103</v>
-      </c>
       <c r="C8" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>108</v>
-      </c>
       <c r="G8" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>117</v>
-      </c>
       <c r="E9" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G9" s="27">
         <v>46323</v>
@@ -6572,22 +6584,22 @@
     </row>
     <row r="10" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>124</v>
-      </c>
       <c r="E10" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G10" s="27">
         <v>46324</v>
@@ -6596,22 +6608,22 @@
     </row>
     <row r="11" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B11" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>129</v>
-      </c>
       <c r="D11" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G11" s="27">
         <v>46325</v>
@@ -6620,22 +6632,22 @@
     </row>
     <row r="12" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="D12" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>138</v>
-      </c>
       <c r="E12" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G12" s="27">
         <v>46326</v>
@@ -6644,48 +6656,48 @@
     </row>
     <row r="13" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B13" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="D13" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="D13" s="9" t="s">
-        <v>144</v>
-      </c>
       <c r="E13" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G13" s="27">
         <v>46327</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>147</v>
-      </c>
       <c r="C14" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>150</v>
-      </c>
       <c r="E14" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G14" s="27">
         <v>46328</v>
@@ -6694,22 +6706,22 @@
     </row>
     <row r="15" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="C15" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="C15" s="9" t="s">
-        <v>154</v>
-      </c>
       <c r="D15" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G15" s="27">
         <v>46329</v>
@@ -6718,22 +6730,22 @@
     </row>
     <row r="16" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B16" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="D16" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>161</v>
-      </c>
       <c r="E16" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G16" s="27">
         <v>46330</v>
@@ -6742,22 +6754,22 @@
     </row>
     <row r="17" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="C17" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="D17" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>166</v>
-      </c>
       <c r="E17" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G17" s="27">
         <v>46331</v>
@@ -6766,22 +6778,22 @@
     </row>
     <row r="18" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="C18" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>169</v>
-      </c>
       <c r="D18" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G18" s="27">
         <v>46332</v>
@@ -6790,22 +6802,22 @@
     </row>
     <row r="19" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B19" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="C19" s="9" t="s">
-        <v>176</v>
-      </c>
       <c r="D19" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G19" s="27">
         <v>46333</v>
@@ -6814,22 +6826,22 @@
     </row>
     <row r="20" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="C20" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>181</v>
-      </c>
       <c r="D20" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G20" s="27">
         <v>46334</v>
@@ -6838,22 +6850,22 @@
     </row>
     <row r="21" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="C21" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="D21" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>188</v>
-      </c>
       <c r="E21" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G21" s="27">
         <v>46335</v>
@@ -6862,22 +6874,22 @@
     </row>
     <row r="22" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="D22" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>195</v>
-      </c>
       <c r="E22" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G22" s="27">
         <v>46336</v>
@@ -6886,22 +6898,22 @@
     </row>
     <row r="23" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="C23" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>199</v>
-      </c>
       <c r="D23" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G23" s="27">
         <v>46337</v>
@@ -6910,22 +6922,22 @@
     </row>
     <row r="24" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B24" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B24" s="9" t="s">
-        <v>210</v>
-      </c>
       <c r="C24" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>213</v>
-      </c>
       <c r="E24" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G24" s="27">
         <v>46338</v>
@@ -6934,22 +6946,22 @@
     </row>
     <row r="25" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B25" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>215</v>
-      </c>
       <c r="C25" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="D25" s="9" t="s">
-        <v>218</v>
-      </c>
       <c r="E25" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G25" s="27">
         <v>46339</v>
@@ -6958,22 +6970,22 @@
     </row>
     <row r="26" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="C26" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="C26" s="9" t="s">
-        <v>222</v>
-      </c>
       <c r="D26" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G26" s="27">
         <v>46340</v>
@@ -6982,22 +6994,22 @@
     </row>
     <row r="27" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B27" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="D27" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="D27" s="9" t="s">
-        <v>229</v>
-      </c>
       <c r="E27" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G27" s="27">
         <v>46341</v>
@@ -7006,22 +7018,22 @@
     </row>
     <row r="28" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C28" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="D28" s="9" t="s">
-        <v>236</v>
-      </c>
       <c r="E28" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G28" s="27">
         <v>46342</v>
@@ -7030,22 +7042,22 @@
     </row>
     <row r="29" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G29" s="27">
         <v>46343</v>
@@ -7054,48 +7066,48 @@
     </row>
     <row r="30" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B30" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="B30" s="9" t="s">
-        <v>243</v>
-      </c>
       <c r="C30" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="D30" s="9" t="s">
-        <v>246</v>
-      </c>
       <c r="E30" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G30" s="27">
         <v>46344</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C31" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="D31" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>251</v>
-      </c>
       <c r="E31" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G31" s="27">
         <v>46345</v>
@@ -7104,22 +7116,22 @@
     </row>
     <row r="32" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="D32" s="9" t="s">
-        <v>256</v>
-      </c>
       <c r="E32" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G32" s="27">
         <v>46346</v>
@@ -7128,74 +7140,74 @@
     </row>
     <row r="33" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C33" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="D33" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="D33" s="9" t="s">
-        <v>260</v>
-      </c>
       <c r="E33" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G33" s="27">
         <v>46347</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="D34" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>265</v>
-      </c>
       <c r="E34" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G34" s="27">
         <v>46348</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C35" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="D35" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="D35" s="9" t="s">
-        <v>270</v>
-      </c>
       <c r="E35" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G35" s="27">
         <v>46349</v>
@@ -7204,22 +7216,22 @@
     </row>
     <row r="36" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="D36" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>274</v>
-      </c>
       <c r="E36" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G36" s="27">
         <v>46350</v>
@@ -7228,22 +7240,22 @@
     </row>
     <row r="37" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="B37" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="C37" s="9" t="s">
+      <c r="D37" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="D37" s="9" t="s">
-        <v>281</v>
-      </c>
       <c r="E37" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G37" s="27">
         <v>46351</v>
@@ -7252,74 +7264,74 @@
     </row>
     <row r="38" spans="1:8" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C38" s="9" t="s">
         <v>285</v>
       </c>
-      <c r="B38" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>287</v>
-      </c>
       <c r="D38" s="9" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G38" s="27">
         <v>46352</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C39" s="9" t="s">
+        <v>292</v>
+      </c>
+      <c r="D39" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="D39" s="9" t="s">
-        <v>296</v>
-      </c>
       <c r="E39" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G39" s="27">
         <v>46353</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C40" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="D40" s="9" t="s">
         <v>302</v>
       </c>
-      <c r="D40" s="9" t="s">
-        <v>304</v>
-      </c>
       <c r="E40" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G40" s="27">
         <v>46354</v>
@@ -7328,22 +7340,22 @@
     </row>
     <row r="41" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C41" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="D41" s="9" t="s">
         <v>308</v>
       </c>
-      <c r="D41" s="9" t="s">
-        <v>310</v>
-      </c>
       <c r="E41" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G41" s="27">
         <v>46355</v>
@@ -7352,22 +7364,22 @@
     </row>
     <row r="42" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G42" s="27">
         <v>46356</v>
@@ -7376,22 +7388,22 @@
     </row>
     <row r="43" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G43" s="27">
         <v>46357</v>
@@ -7400,22 +7412,22 @@
     </row>
     <row r="44" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C44" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="D44" s="9" t="s">
         <v>334</v>
       </c>
-      <c r="D44" s="9" t="s">
-        <v>336</v>
-      </c>
       <c r="E44" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G44" s="27">
         <v>46358</v>
@@ -7424,22 +7436,22 @@
     </row>
     <row r="45" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G45" s="27">
         <v>46359</v>
@@ -7448,22 +7460,22 @@
     </row>
     <row r="46" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C46" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="D46" s="9" t="s">
         <v>352</v>
       </c>
-      <c r="D46" s="9" t="s">
-        <v>354</v>
-      </c>
       <c r="E46" s="8" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G46" s="27">
         <v>46360</v>
@@ -7472,22 +7484,22 @@
     </row>
     <row r="47" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C47" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="D47" s="9" t="s">
         <v>362</v>
       </c>
-      <c r="D47" s="9" t="s">
-        <v>364</v>
-      </c>
       <c r="E47" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G47" s="27">
         <v>46361</v>
@@ -7496,22 +7508,22 @@
     </row>
     <row r="48" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G48" s="27">
         <v>46362</v>
@@ -7520,22 +7532,22 @@
     </row>
     <row r="49" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A49" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C49" s="9" t="s">
         <v>378</v>
       </c>
-      <c r="B49" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="C49" s="9" t="s">
+      <c r="D49" s="9" t="s">
         <v>380</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>382</v>
-      </c>
       <c r="E49" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G49" s="27">
         <v>46363</v>
@@ -7544,22 +7556,22 @@
     </row>
     <row r="50" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G50" s="27">
         <v>46364</v>
@@ -7568,54 +7580,54 @@
     </row>
     <row r="51" spans="1:8" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G51" s="27">
         <v>46365</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="165.6" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C52" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="D52" s="9" t="s">
         <v>398</v>
       </c>
-      <c r="D52" s="9" t="s">
-        <v>400</v>
-      </c>
       <c r="E52" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G52" s="27">
         <v>46366</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
   </sheetData>
@@ -7641,23 +7653,23 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
@@ -7665,22 +7677,22 @@
     </row>
     <row r="5" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="13" t="s">
-        <v>63</v>
-      </c>
       <c r="E5" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>65</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -7711,48 +7723,48 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>103</v>
-      </c>
       <c r="C8" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>108</v>
-      </c>
       <c r="G8" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G9" s="27">
         <v>46323</v>
@@ -7761,22 +7773,22 @@
     </row>
     <row r="10" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>293</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>295</v>
-      </c>
       <c r="E10" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G10" s="27">
         <v>46323</v>
@@ -7785,22 +7797,22 @@
     </row>
     <row r="11" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>300</v>
-      </c>
       <c r="D11" s="9" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G11" s="27">
         <v>46323</v>
@@ -7809,22 +7821,22 @@
     </row>
     <row r="12" spans="1:8" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C12" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>311</v>
-      </c>
       <c r="E12" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G12" s="27">
         <v>46323</v>
@@ -7833,22 +7845,22 @@
     </row>
     <row r="13" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B13" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>469</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>471</v>
-      </c>
       <c r="D13" s="9" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G13" s="27">
         <v>46323</v>
@@ -7857,22 +7869,22 @@
     </row>
     <row r="14" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G14" s="27">
         <v>46323</v>
@@ -7881,48 +7893,48 @@
     </row>
     <row r="15" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G15" s="27">
         <v>46323</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G16" s="27">
         <v>46323</v>
@@ -7931,22 +7943,22 @@
     </row>
     <row r="17" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G17" s="27">
         <v>46323</v>
@@ -7955,22 +7967,22 @@
     </row>
     <row r="18" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G18" s="27">
         <v>46323</v>
@@ -7979,22 +7991,22 @@
     </row>
     <row r="19" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C19" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>363</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>365</v>
-      </c>
       <c r="E19" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G19" s="27">
         <v>46323</v>
@@ -8003,22 +8015,22 @@
     </row>
     <row r="20" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G20" s="27">
         <v>46323</v>
@@ -8027,22 +8039,22 @@
     </row>
     <row r="21" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C21" s="9" t="s">
+        <v>379</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>381</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>383</v>
-      </c>
       <c r="E21" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G21" s="27">
         <v>46323</v>
@@ -8051,22 +8063,22 @@
     </row>
     <row r="22" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G22" s="27">
         <v>46323</v>
@@ -8075,22 +8087,22 @@
     </row>
     <row r="23" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C23" s="9" t="s">
+        <v>392</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>394</v>
       </c>
-      <c r="D23" s="9" t="s">
-        <v>396</v>
-      </c>
       <c r="E23" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G23" s="27">
         <v>46323</v>
@@ -8099,48 +8111,48 @@
     </row>
     <row r="24" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G24" s="27">
         <v>46323</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>403</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>404</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>405</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>406</v>
-      </c>
       <c r="E25" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G25" s="27">
         <v>46323</v>
@@ -8149,22 +8161,22 @@
     </row>
     <row r="26" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
+        <v>405</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>409</v>
-      </c>
       <c r="D26" s="9" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G26" s="27">
         <v>46323</v>
@@ -8173,22 +8185,22 @@
     </row>
     <row r="27" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>413</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>415</v>
-      </c>
       <c r="D27" s="9" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G27" s="27">
         <v>46323</v>
@@ -8197,22 +8209,22 @@
     </row>
     <row r="28" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
+        <v>416</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>418</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>420</v>
-      </c>
       <c r="D28" s="9" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G28" s="27">
         <v>46323</v>
@@ -8237,16 +8249,16 @@
     <col min="5" max="5" width="24.21875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" customWidth="1"/>
     <col min="9" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G2" s="21" t="s">
         <v>4</v>
@@ -8254,15 +8266,15 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
@@ -8270,36 +8282,36 @@
     </row>
     <row r="5" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="13" t="s">
-        <v>63</v>
-      </c>
       <c r="E5" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>65</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="16">
         <f>COUNTIF(F9:F28, "Passed")</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B6" s="17">
         <f>COUNTIF(F9:F28, "Failed")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C6" s="18">
         <f>COUNTBLANK(F9:F28) + COUNTIF(F9:F28, "Untested")</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D6" s="19">
         <f>COUNTIF(F9:F28, "Blocked")</f>
@@ -8316,428 +8328,516 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>103</v>
-      </c>
       <c r="C8" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>108</v>
-      </c>
       <c r="G8" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>323</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>325</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>327</v>
-      </c>
       <c r="E9" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
+        <v>118</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="27">
+        <v>46324</v>
+      </c>
       <c r="H9" s="9"/>
     </row>
     <row r="10" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>312</v>
-      </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+        <v>310</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="27">
+        <v>46324</v>
+      </c>
       <c r="H10" s="9"/>
     </row>
     <row r="11" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>340</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>244</v>
-      </c>
-      <c r="C11" s="9" t="s">
+      <c r="D11" s="9" t="s">
         <v>342</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>344</v>
-      </c>
       <c r="E11" s="8" t="s">
-        <v>312</v>
-      </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+        <v>310</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="27">
+        <v>46324</v>
+      </c>
       <c r="H11" s="9"/>
     </row>
     <row r="12" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>312</v>
-      </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+        <v>310</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" s="27">
+        <v>46324</v>
+      </c>
       <c r="H12" s="9"/>
     </row>
     <row r="13" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>312</v>
-      </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+        <v>310</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="27">
+        <v>46324</v>
+      </c>
       <c r="H13" s="9"/>
     </row>
     <row r="14" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>312</v>
-      </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+        <v>310</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" s="27">
+        <v>46324</v>
+      </c>
       <c r="H14" s="9"/>
     </row>
     <row r="15" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>312</v>
-      </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
+        <v>310</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" s="27">
+        <v>46324</v>
+      </c>
       <c r="H15" s="9"/>
     </row>
     <row r="16" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+        <v>371</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G16" s="27">
+        <v>46324</v>
+      </c>
       <c r="H16" s="9"/>
     </row>
     <row r="17" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="D17" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G17" s="27">
+        <v>46324</v>
+      </c>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
         <v>412</v>
       </c>
-      <c r="E17" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="9"/>
-    </row>
-    <row r="18" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
-        <v>414</v>
-      </c>
       <c r="B18" s="9" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C18" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>417</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>419</v>
-      </c>
       <c r="E18" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="9"/>
-    </row>
-    <row r="19" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
+        <v>371</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" s="27">
+        <v>46324</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>422</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>268</v>
-      </c>
-      <c r="C19" s="9" t="s">
+      <c r="E19" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="27">
+        <v>46324</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
         <v>423</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="B20" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>424</v>
       </c>
-      <c r="E19" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="9"/>
-    </row>
-    <row r="20" spans="1:8" ht="69" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
+      <c r="D20" s="9" t="s">
         <v>425</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="C20" s="9" t="s">
+      <c r="E20" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G20" s="27">
+        <v>46324</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
         <v>426</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="B21" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>427</v>
       </c>
-      <c r="E20" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="9"/>
-    </row>
-    <row r="21" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="8" t="s">
+      <c r="D21" s="9" t="s">
         <v>428</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>429</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>430</v>
-      </c>
       <c r="E21" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="9"/>
+        <v>371</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" s="27">
+        <v>46324</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>475</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>431</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>432</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>433</v>
-      </c>
       <c r="E22" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
+        <v>371</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G22" s="27">
+        <v>46324</v>
+      </c>
       <c r="H22" s="9"/>
     </row>
     <row r="23" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>284</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>434</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>286</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>435</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>436</v>
-      </c>
       <c r="E23" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+        <v>371</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G23" s="27">
+        <v>46324</v>
+      </c>
       <c r="H23" s="9"/>
     </row>
     <row r="24" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
+        <v>435</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>437</v>
       </c>
-      <c r="B24" s="9" t="s">
-        <v>292</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>438</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>439</v>
-      </c>
       <c r="E24" s="8" t="s">
-        <v>387</v>
-      </c>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
+        <v>385</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G24" s="27">
+        <v>46324</v>
+      </c>
       <c r="H24" s="9"/>
     </row>
     <row r="25" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
+        <v>438</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>297</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>441</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>442</v>
-      </c>
       <c r="E25" s="8" t="s">
-        <v>387</v>
-      </c>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
+        <v>385</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G25" s="27">
+        <v>46324</v>
+      </c>
       <c r="H25" s="9"/>
     </row>
     <row r="26" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
+        <v>441</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>443</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>444</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>445</v>
-      </c>
       <c r="E26" s="8" t="s">
-        <v>437</v>
-      </c>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
+        <v>435</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G26" s="27">
+        <v>46324</v>
+      </c>
       <c r="H26" s="9"/>
     </row>
     <row r="27" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>446</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>316</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>447</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>448</v>
-      </c>
       <c r="E27" s="8" t="s">
-        <v>387</v>
-      </c>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
+        <v>385</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G27" s="27">
+        <v>46324</v>
+      </c>
       <c r="H27" s="9"/>
     </row>
     <row r="28" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>448</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>449</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>324</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>450</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>451</v>
-      </c>
       <c r="E28" s="8" t="s">
-        <v>387</v>
-      </c>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
+        <v>385</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G28" s="27">
+        <v>46324</v>
+      </c>
       <c r="H28" s="9"/>
     </row>
   </sheetData>
@@ -8761,7 +8861,7 @@
   <sheetData>
     <row r="2" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B2" s="28" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C2" s="29"/>
       <c r="D2" s="29"/>
@@ -8804,7 +8904,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>12</v>
@@ -8815,10 +8915,10 @@
     </row>
     <row r="7" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>16</v>
@@ -8832,25 +8932,25 @@
         <v>27</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="F10" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>457</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>458</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
@@ -8858,7 +8958,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D11" s="8">
         <f>'Admin - Orders'!A6</f>
@@ -8890,7 +8990,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D12" s="8">
         <f>'Admin - Shipments'!A6</f>
@@ -8922,19 +9022,19 @@
         <v>3</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D13" s="8">
         <f>'Admin - Gift cards'!A6</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E13" s="8">
         <f>'Admin - Gift cards'!B6</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F13" s="8">
         <f>'Admin - Gift cards'!C6</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G13" s="8">
         <f>'Admin - Gift cards'!D6</f>
@@ -8951,19 +9051,19 @@
     </row>
     <row r="14" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C14" s="24" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="D14" s="13">
         <f t="shared" ref="D14:I14" si="0">SUM(D11:D13)</f>
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="E14" s="13">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F14" s="13">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G14" s="13">
         <f t="shared" si="0"/>
@@ -8980,26 +9080,26 @@
     </row>
     <row r="16" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C16" s="25" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="E16" s="26">
         <f>IF(I14-H14=0, 0, (D14+E14)/(I14-H14)*100)</f>
-        <v>73.80952380952381</v>
+        <v>97.61904761904762</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="17" spans="3:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C17" s="25" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="E17" s="26">
         <f>IF(D14+E14=0, 0, D14/(D14+E14)*100)</f>
-        <v>88.709677419354833</v>
+        <v>86.58536585365853</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="21" spans="3:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>